<commit_message>
feat(rd-jachymov): sklad S01/S03a přepočet + zásyp/plot/zábradlí položky
Geometrie upřesněna dle ručního obmeru + řezů (uživatel):
- S01 podlaha: 17.6 m² (místnost) + 6.0 (vynos za stěnu, řez B-B) = 23.6 m²
  · HSV1.005 podkladní drť 150mm 2.64→3.54 m³
  · PSV77.001 dlažba 17.6→23.6 m²
  · NEW HSV1.007 kladecí lože drť 40mm 0.94 m³ (vrstva dříve chyběla)
- S03a tvárnice: výška 14 řad×250 = 3.5 m (PLNÁ, od pasu; 2.68 je světlá)
  · HSV3.002 46.5→62.5 m² (3 strany 17.84 m × 3.5)
  · HSV3.003 výztuž 1398→1875 kg
- NEW položky (geometrie známa, materiál OVĚŘIT → queue #36-38):
  · HSV1.008 zásyp za prefa stěnou 23.5 m³ (#36)
  · PSV76.003 oplocení 3.8 bm (#37)
  · PSV76.004 zábradlí 18.5 bm (#38)

queue 31→34; docx==queue assertion OK; 0 duplicitních ID (238 položek)

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/ATOMIC_FLAT_2026-06-02.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/ATOMIC_FLAT_2026-06-02.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ATOMIC_FLAT" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ATOMIC_FLAT'!$A$1:$M$361</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ATOMIC_FLAT'!$A$1:$M$366</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M361"/>
+  <dimension ref="A1:M366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1714,11 +1714,11 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>2.64</v>
+        <v>3.54</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>podlaha sklad 17.6 m² (legenda místností) × 0.15 m podkladní kamenná drť</t>
+          <t>S01 plocha 23.6 m² (místnost 17.6 + vynos za stěnu 6.0 dle řezu) × 0.15 m podkladní drť 4-8 = 3.54 m³</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>DXF podlaha skladu 6.35×3.34 = 21.2 m²</t>
+          <t>legenda místností 17.6 m² + vynos S01 za stěnu 6010×1000 mm dle řezu B-B (neviditelný na půdorysu)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Montáž — Obvodové stěny skladu — tvarovky ztraceného bednění tl. 250 mm × výška 2.4 m + zalití C25/30</t>
+          <t>Montáž — Obvodové stěny skladu S03a/b — tvarovky ztraceného bednění tl. 250 mm, výška 14 řad × 250 = 3.5 m + zalití C25/30</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -4018,11 +4018,11 @@
         </is>
       </c>
       <c r="H60" s="2" t="n">
-        <v>46.5</v>
+        <v>62.5</v>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>obvod 19.4 m × výška 2.4 m = 46.6</t>
+          <t>3 strany trapézu (6010-1000 dveře)+(7000-600 prefa)+(7033-600 prefa)=17843 mm = 17.84 m × výška 14 řad×0.25 = 3.5 m = 62.5 m²</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>TZ statika sklad §4 + DXF DIMENSION obvod</t>
+          <t>výkres D.1.1.02/03 — 14 řad tvárnic × 250 mm (řady začínají pod úrovní podlahy od pasu); světlá 2.68 je vnitřní svět, NE výška tvárnic</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Dodávka — Pronájem bednění (Obvodové stěny skladu — tvarovky ztraceného be)</t>
+          <t>Dodávka — Pronájem bednění (Obvodové stěny skladu S03a/b — tvarovky ztrace)</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -4081,7 +4081,7 @@
         </is>
       </c>
       <c r="H61" s="2" t="n">
-        <v>46.5</v>
+        <v>62.5</v>
       </c>
       <c r="I61" s="3">
         <f> montáž 1:1</f>
@@ -4090,7 +4090,7 @@
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>TZ statika sklad §4 + DXF DIMENSION obvod</t>
+          <t>výkres D.1.1.02/03 — 14 řad tvárnic × 250 mm (řady začínají pod úrovní podlahy od pasu); světlá 2.68 je vnitřní svět, NE výška tvárnic</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
@@ -4139,11 +4139,11 @@
         </is>
       </c>
       <c r="H62" s="2" t="n">
-        <v>1398</v>
+        <v>1875</v>
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>46.6 × 30 kg/m² = 1398</t>
+          <t>62.5 m² × 30 kg/m² (zalití C25/30) = 1875 kg</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -4151,10 +4151,9 @@
           <t>273361821</t>
         </is>
       </c>
-      <c r="K62" s="3" t="inlineStr">
-        <is>
-          <t>B4_productivity Methvin — výztuž do ZB tvarovek tl. 250 mm</t>
-        </is>
+      <c r="K62" s="3">
+        <f> HSV3.002 plocha (62.5 m²) × 30 kg/m²</f>
+        <v/>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
@@ -4202,17 +4201,16 @@
         </is>
       </c>
       <c r="H63" s="2" t="n">
-        <v>1398</v>
+        <v>1875</v>
       </c>
       <c r="I63" s="3">
         <f> montáž 1:1</f>
         <v/>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
-      <c r="K63" s="3" t="inlineStr">
-        <is>
-          <t>B4_productivity Methvin — výztuž do ZB tvarovek tl. 250 mm</t>
-        </is>
+      <c r="K63" s="3">
+        <f> HSV3.002 plocha (62.5 m²) × 30 kg/m²</f>
+        <v/>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
@@ -13739,7 +13737,7 @@
       </c>
       <c r="F226" s="3" t="inlineStr">
         <is>
-          <t>Betonová dlažba do pískového lože — povrch podlahy skladu (~21 m²)</t>
+          <t>Betonová dlažba 50 mm do kladecího lože — podlaha skladu + vynos za stěnu</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -13748,17 +13746,17 @@
         </is>
       </c>
       <c r="H226" s="2" t="n">
-        <v>17.6</v>
+        <v>23.6</v>
       </c>
       <c r="I226" s="3" t="inlineStr">
         <is>
-          <t>DXF sklad_DPZ km_tabulka místností room 0.01 (sklad zahradní techniky) = 17.60 m² (inner usable area per DXF room table, walls excluded). Prior estimate 21.209 m² (outer 6.35×3.34) over-counted by 17.0% — walls of tvarovky ZB tl. 250 mm take ~3.6 m² of outer footprint.</t>
+          <t>plocha S01 = místnost 17.6 (legenda) + vynos za stěnu 6.0 (6010×1000 řez) = 23.6 m²</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr"/>
       <c r="K226" s="3" t="inlineStr">
         <is>
-          <t>DXF sklad_DPZ km_tabulka místností + Phase 3.5 sklad qty crosscheck (Pattern 17 Phase 0a Layer 2 + Pattern 31 CEV Matrix D.2)</t>
+          <t>legenda místností 17.6 + vynos S01 za stěnu (řez B-B)</t>
         </is>
       </c>
       <c r="L226" s="2" t="inlineStr">
@@ -21604,8 +21602,294 @@
         </is>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" s="2" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" s="2" t="inlineStr">
+        <is>
+          <t>HSV1.007</t>
+        </is>
+      </c>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>260217_sklad</t>
+        </is>
+      </c>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>HSV-1 Zemní práce</t>
+        </is>
+      </c>
+      <c r="E362" s="3" t="inlineStr">
+        <is>
+          <t>HSV-1 Zemní práce</t>
+        </is>
+      </c>
+      <c r="F362" s="3" t="inlineStr">
+        <is>
+          <t>Kladecí lože z kamenné drti 4-8 mm tl. 40 mm pod betonovou dlažbu skladu</t>
+        </is>
+      </c>
+      <c r="G362" s="2" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="H362" s="2" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="I362" s="3" t="inlineStr">
+        <is>
+          <t>S01 plocha 23.6 m² × 0.04 m = 0.94 m³</t>
+        </is>
+      </c>
+      <c r="J362" s="2" t="inlineStr">
+        <is>
+          <t>564231111</t>
+        </is>
+      </c>
+      <c r="K362" s="3" t="inlineStr">
+        <is>
+          <t>skladba S01 — kladecí vrstva kamenná drť 4-8 mm 40 mm (vrstva dříve chyběla)</t>
+        </is>
+      </c>
+      <c r="L362" s="2" t="inlineStr">
+        <is>
+          <t>needs_production_lookup</t>
+        </is>
+      </c>
+      <c r="M362" s="2" t="inlineStr">
+        <is>
+          <t>S01_sklad</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" s="2" t="inlineStr">
+        <is>
+          <t>HSV1.008</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>260217_sklad</t>
+        </is>
+      </c>
+      <c r="D363" s="2" t="inlineStr">
+        <is>
+          <t>HSV-1 Zemní práce</t>
+        </is>
+      </c>
+      <c r="E363" s="3" t="inlineStr">
+        <is>
+          <t>HSV-1 Zemní práce</t>
+        </is>
+      </c>
+      <c r="F363" s="3" t="inlineStr">
+        <is>
+          <t>Zásyp za prefabrikovanou opěrnou stěnou S04 — materiál dle PD (NEuveden v legendě, OVĚŘIT)</t>
+        </is>
+      </c>
+      <c r="G363" s="2" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="H363" s="2" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="I363" s="3" t="inlineStr">
+        <is>
+          <t>průřez zásypu 3.61 m² (řez A-A) × délka 6.5 m = 23.5 m³</t>
+        </is>
+      </c>
+      <c r="J363" s="2" t="inlineStr">
+        <is>
+          <t>174101101</t>
+        </is>
+      </c>
+      <c r="K363" s="3" t="inlineStr">
+        <is>
+          <t>řez A-A — klín zásypu za S04; materiál v legendě NEuveden → OVĚŘIT</t>
+        </is>
+      </c>
+      <c r="L363" s="2" t="inlineStr">
+        <is>
+          <t>needs_production_lookup</t>
+        </is>
+      </c>
+      <c r="M363" s="2" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" s="2" t="inlineStr">
+        <is>
+          <t>PSV76.003</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>260217_sklad</t>
+        </is>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>PSV-76 Zámečnické konstrukce</t>
+        </is>
+      </c>
+      <c r="E364" s="3" t="inlineStr">
+        <is>
+          <t>PSV-76 Zámečnické konstrukce</t>
+        </is>
+      </c>
+      <c r="F364" s="3" t="inlineStr">
+        <is>
+          <t>Oplocení podél vjezdu — délka dle situace, materiál OVĚŘIT (kov/dřevo neuveden)</t>
+        </is>
+      </c>
+      <c r="G364" s="2" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H364" s="2" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="I364" s="3" t="inlineStr">
+        <is>
+          <t>šířka 7775 − 4000 (posuvná vrata) = 3775 mm ≈ 3.8 bm</t>
+        </is>
+      </c>
+      <c r="J364" s="2" t="inlineStr"/>
+      <c r="K364" s="3" t="inlineStr">
+        <is>
+          <t>D.1.1.01 půdorys střechy — plot u vjezdu; materiál + přesná délka OVĚŘIT</t>
+        </is>
+      </c>
+      <c r="L364" s="2" t="inlineStr">
+        <is>
+          <t>needs_production_lookup</t>
+        </is>
+      </c>
+      <c r="M364" s="2" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" s="2" t="inlineStr">
+        <is>
+          <t>PSV76.004a</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>260217_sklad</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>PSV-76 Zámečnické konstrukce</t>
+        </is>
+      </c>
+      <c r="E365" s="3" t="inlineStr">
+        <is>
+          <t>PSV-76 Zámečnické konstrukce</t>
+        </is>
+      </c>
+      <c r="F365" s="3" t="inlineStr">
+        <is>
+          <t>Montáž — Zábradlí v. 1.0 m kolem části stání — materiál OVĚŘIT (kov/dřevo neuveden)</t>
+        </is>
+      </c>
+      <c r="G365" s="2" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H365" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I365" s="3" t="inlineStr">
+        <is>
+          <t>obvod části stání ≈ 18.5 bm (D.1.1.01), výška 1.0 m</t>
+        </is>
+      </c>
+      <c r="J365" s="2" t="inlineStr"/>
+      <c r="K365" s="3" t="inlineStr">
+        <is>
+          <t>D.1.1.01 — zábradlí 1.0 m kolem části plochy; materiál OVĚŘIT</t>
+        </is>
+      </c>
+      <c r="L365" s="2" t="inlineStr">
+        <is>
+          <t>needs_production_lookup</t>
+        </is>
+      </c>
+      <c r="M365" s="2" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" s="2" t="inlineStr">
+        <is>
+          <t>PSV76.004b</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>260217_sklad</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>PSV-76 Zámečnické konstrukce</t>
+        </is>
+      </c>
+      <c r="E366" s="3" t="inlineStr">
+        <is>
+          <t>PSV-76 Zámečnické konstrukce</t>
+        </is>
+      </c>
+      <c r="F366" s="3" t="inlineStr">
+        <is>
+          <t>Dodávka — Dodávka výrobku (Zábradlí v. 1.0 m kolem části stání — materiál)</t>
+        </is>
+      </c>
+      <c r="G366" s="2" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H366" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I366" s="3">
+        <f> montáž 1:1</f>
+        <v/>
+      </c>
+      <c r="J366" s="2" t="inlineStr"/>
+      <c r="K366" s="3" t="inlineStr">
+        <is>
+          <t>D.1.1.01 — zábradlí 1.0 m kolem části plochy; materiál OVĚŘIT</t>
+        </is>
+      </c>
+      <c r="L366" s="2" t="inlineStr">
+        <is>
+          <t>needs_lookup</t>
+        </is>
+      </c>
+      <c r="M366" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M361"/>
+  <autoFilter ref="A1:M366"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(rd-jachymov): sklad základy — bednění + výztuž patek/pasů + věnec 6.7
Uživatel: ztracené bednění z tvárnic = duté bloky zalité betonem + výztuž
uvnitř; chyběla opalubka + výztuž patek a pasů.
- HSV2.007 NEW bednění základů (patky spodní 6 m² + pasy 19.4 m²) = 25.4 m²
- HSV2.008 NEW výztuž B500B do tvárnic ZB (patky horní + věnec) = 153 kg
  (zálivka 1.275 m³ × 120 kg/m³ = stěna 30 kg/m² ÷ 0.25)
- HSV2.004 věnec délka 6.35→6.7 m (ruční obmer), zálivka → 1.77 m³
- queue #42: bednění do rýhy vs systémové + prostý beton pasů (výztuž?) OVĚŘIT

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/ATOMIC_FLAT_2026-06-02.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/ATOMIC_FLAT_2026-06-02.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ATOMIC_FLAT" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ATOMIC_FLAT'!$A$1:$M$372</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ATOMIC_FLAT'!$A$1:$M$374</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M372"/>
+  <dimension ref="A1:M374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3106,11 +3106,11 @@
         </is>
       </c>
       <c r="H45" s="2" t="n">
-        <v>1.75</v>
+        <v>1.77</v>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>patky horní (0.3×0.3×0.5×6 = 0.27) + věnec nad patkami 2 řady ztrac.bednění (0.5 v × 6.35 d × 0.3 š = 0.95) + zídka lemující (~0.5) = ~1.72 ≈ 1.75 m³</t>
+          <t>zálivka tvárnic ZB: patky horní (0.3×0.3×0.5×6=0.27) + věnec 2 řady (2×0.25 v × 0.3 š × 6.7 d=1.00) + zídka lemující (~0.5) = 1.77 m³</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>TZ statika sklad §3 + výkres D.1.1.02 — věnec 2 řady nad 6 patkami, šířka tvárnic 300 mm</t>
+          <t>TZ statika sklad §3 + výkres D.1.1.02 — věnec délka 6.7 m (ruční obmer)</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -22236,8 +22236,126 @@
         </is>
       </c>
     </row>
+    <row r="373">
+      <c r="A373" s="2" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" s="2" t="inlineStr">
+        <is>
+          <t>HSV2.007</t>
+        </is>
+      </c>
+      <c r="C373" s="2" t="inlineStr">
+        <is>
+          <t>260217_sklad</t>
+        </is>
+      </c>
+      <c r="D373" s="2" t="inlineStr">
+        <is>
+          <t>HSV-2 Základové a ŽB</t>
+        </is>
+      </c>
+      <c r="E373" s="3" t="inlineStr">
+        <is>
+          <t>HSV-2 Základové a ŽB</t>
+        </is>
+      </c>
+      <c r="F373" s="3" t="inlineStr">
+        <is>
+          <t>Bednění základových pasů + spodních patek (prostý beton) — tradiční / systémové, oboustranné kde nelze betonovat do rýhy</t>
+        </is>
+      </c>
+      <c r="G373" s="2" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="H373" s="2" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="I373" s="3" t="inlineStr">
+        <is>
+          <t>patky spodní 6×4×0.5×0.5=6.0 + pasy 2 strany×0.5×19.4 obvod=19.4 = 25.4 m² (část lze betonovat do rýhy → OVĚŘIT)</t>
+        </is>
+      </c>
+      <c r="J373" s="2" t="inlineStr">
+        <is>
+          <t>273351215</t>
+        </is>
+      </c>
+      <c r="K373" s="3" t="inlineStr">
+        <is>
+          <t>výkres D.1.1.02 + řez — bednění základů; podíl do rýhy vs systémové OVĚŘIT</t>
+        </is>
+      </c>
+      <c r="L373" s="2" t="inlineStr">
+        <is>
+          <t>needs_production_lookup</t>
+        </is>
+      </c>
+      <c r="M373" s="2" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" s="2" t="inlineStr">
+        <is>
+          <t>HSV2.008</t>
+        </is>
+      </c>
+      <c r="C374" s="2" t="inlineStr">
+        <is>
+          <t>260217_sklad</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>HSV-2 Základové a ŽB</t>
+        </is>
+      </c>
+      <c r="E374" s="3" t="inlineStr">
+        <is>
+          <t>HSV-2 Základové a ŽB</t>
+        </is>
+      </c>
+      <c r="F374" s="3" t="inlineStr">
+        <is>
+          <t>Výztuž B500B vkládaná do tvárnic ztraceného bednění — patky horní (6 sloupků) + ztužující věnec nad patkami</t>
+        </is>
+      </c>
+      <c r="G374" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="H374" s="2" t="n">
+        <v>153</v>
+      </c>
+      <c r="I374" s="3" t="inlineStr">
+        <is>
+          <t>zálivka tvárnic ZB 1.27 m³ (patky horní 0.27 + věnec 1.00) × 120 kg/m³ (= stěna 30 kg/m² ÷ 0.25) = 153 kg</t>
+        </is>
+      </c>
+      <c r="J374" s="2" t="inlineStr">
+        <is>
+          <t>273361821</t>
+        </is>
+      </c>
+      <c r="K374" s="3" t="inlineStr">
+        <is>
+          <t>TZ statika sklad §3 — výztuž B500B do tvárnic ZB; sazba dle stěny S03a (HSV3.003)</t>
+        </is>
+      </c>
+      <c r="L374" s="2" t="inlineStr">
+        <is>
+          <t>needs_production_lookup</t>
+        </is>
+      </c>
+      <c r="M374" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M372"/>
+  <autoFilter ref="A1:M374"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>